<commit_message>
feat: Add Pydantic validation for GenAI agent inputs
- Introduce `VideoAnalysisInput` Pydantic model to strictly validate video metadata.
- Prevent prompt injection by sanitizing titles.
- Enforce constraints on views and retention data.
- Update `GeminiThinkingAgent` to use the validated model.
- Add `tests/test_security_validation.py` to verify security constraints.
</commit_message>
<xml_diff>
--- a/bachata_analytics.xlsx
+++ b/bachata_analytics.xlsx
@@ -447,7 +447,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -483,19 +483,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vid_1</t>
+          <t>vid_16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Basic Step Tutorial</t>
+          <t>Musicality 101</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>445271</v>
+        <v>460541</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>62.35665762978796</v>
+        <v>36.09895327395583</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -518,9 +518,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -554,19 +554,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vid_14</t>
+          <t>vid_6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Advanced Footwork</t>
+          <t>Musicality 101</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>445679</v>
+        <v>441441</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>90.21670767832464</v>
+        <v>89.25828491457786</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -577,19 +577,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>vid_15</t>
+          <t>vid_9</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Partner Connection Secrets</t>
+          <t>Dip Technique</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>440398</v>
+        <v>404774</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>31.99203356798657</v>
+        <v>58.78825956714138</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>